<commit_message>
MU thesis revision: $625 PT base / $1,000+ structural HBM bull. Updates deck, leave-behind, through-cycle long, tear sheets, comps demo, and toolkit XLSX inputs.
</commit_message>
<xml_diff>
--- a/assets/toolkit/MU_ai_cycle.xlsx
+++ b/assets/toolkit/MU_ai_cycle.xlsx
@@ -932,6 +932,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -976,7 +977,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -1004,6 +1005,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
@@ -1012,7 +1014,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Near peak</t>
+          <t>Cycle peak (FY26-27 print, expect normalization)</t>
         </is>
       </c>
     </row>
@@ -1056,6 +1058,7 @@
         <v>-0.1254826254826255</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
@@ -1118,6 +1121,7 @@
         <v/>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
@@ -1130,6 +1134,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
@@ -5669,6 +5674,7 @@
       <c r="B1" s="27" t="n"/>
       <c r="C1" s="22" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -5707,7 +5713,7 @@
         </is>
       </c>
       <c r="B6" s="29" t="n">
-        <v>108.45</v>
+        <v>668</v>
       </c>
     </row>
     <row r="7">
@@ -5730,6 +5736,7 @@
         <v>1.27</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -5746,7 +5753,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="12">
@@ -5844,6 +5851,7 @@
         <v>0.15</v>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
@@ -5913,6 +5921,7 @@
         <v>0.18</v>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
@@ -5942,6 +5951,7 @@
         <v>10</v>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
@@ -6848,9 +6858,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A17:C22"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A17:C22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
ship: Market recap — The Market Is Cooling Under the Semis (May 8, 2026); v=28
</commit_message>
<xml_diff>
--- a/assets/toolkit/MU_ai_cycle.xlsx
+++ b/assets/toolkit/MU_ai_cycle.xlsx
@@ -8,21 +8,22 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drivers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historicals" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cycle Diagnostic" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Statement" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LBO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns Attribution" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M&amp;A" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Football" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reverse-DCF" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reverse-LBO" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sanity Checks" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Sources" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historicals" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cycle Diagnostic" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Statement" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LBO" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns Attribution" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M&amp;A" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Football" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reverse-DCF" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reverse-LBO" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sanity Checks" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="ib_betaT">Drivers!$B$26</definedName>
@@ -78,7 +79,7 @@
     <numFmt numFmtId="170" formatCode="#,##0&quot; bps&quot;"/>
     <numFmt numFmtId="171" formatCode="0.00&quot;×&quot;"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -170,8 +171,35 @@
     <font>
       <i val="1"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF7F2700"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF7F2700"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF7F2700"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFB0432A"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="FF0B3D91"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -250,6 +278,11 @@
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB0432A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -322,7 +355,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -388,6 +421,17 @@
     <xf numFmtId="171" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -918,7 +962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32.7109375" customWidth="1" min="1" max="1"/>
@@ -926,225 +970,246 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="51" t="inlineStr">
+        <is>
+          <t>⚠ DEMO DATA — see 'Data Sources' tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="52" t="inlineStr">
+        <is>
+          <t>Market data was sourced from a synthetic test harness, NOT live yfinance. Re-run `python run_model.py MU` to refresh against live market data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="53" t="inlineStr">
+        <is>
+          <t>Market data as-of: 2026-05-08 02:59 UTC  ·  Source: demo/synthetic</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Micron Technology, Inc. (MU) — IB Valuation Template</t>
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Sector / Industry</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Technology / Semiconductors</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Reporting Currency</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Fiscal Year End</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2025-08-31</t>
-        </is>
-      </c>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>As-of Date</t>
+          <t>Sector / Industry</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>Technology / Semiconductors</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Industry Preset</t>
+          <t>Reporting Currency</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>semiconductors_ai_cycle</t>
+          <t>USD</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Mid-cycle method</t>
+          <t>Fiscal Year End</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>peak_half</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
+          <t>2025-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>As-of Date</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Cycle phase</t>
+          <t>Industry Preset</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cycle peak (FY26-27 print, expect normalization)</t>
+          <t>semiconductors_ai_cycle</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Position in margin range</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>0.9640387710165633</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Latest EBITDA margin</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>0.4647887323943662</v>
-      </c>
-    </row>
+          <t>Mid-cycle method</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>peak_half</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>5y peak margin</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>0.4868074354809601</v>
+          <t>Cycle phase</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Near peak</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>5y trough margin</t>
+          <t>Position in margin range</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>-0.1254826254826255</v>
-      </c>
-    </row>
-    <row r="15"/>
+        <v>0.9640387710165633</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Latest EBITDA margin</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0.4647887323943662</v>
+      </c>
+    </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Headline outputs (linked)</t>
-        </is>
-      </c>
-      <c r="B16" s="22" t="n"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>5y peak margin</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0.4868074354809601</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Current Market Price</t>
-        </is>
-      </c>
-      <c r="B17" s="23" t="n">
-        <v>108.45</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>DCF Implied Price</t>
-        </is>
-      </c>
-      <c r="B18" s="24">
-        <f>DCF!B40</f>
-        <v/>
-      </c>
-    </row>
+          <t>5y trough margin</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>-0.1254826254826255</v>
+      </c>
+    </row>
+    <row r="18"/>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>DCF Upside / (Downside)</t>
-        </is>
-      </c>
-      <c r="B19" s="25">
-        <f>B18/B17-1</f>
-        <v/>
-      </c>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Headline outputs (linked)</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>LBO Sponsor IRR</t>
-        </is>
-      </c>
-      <c r="B20" s="25">
-        <f>LBO!B40</f>
-        <v/>
+          <t>Current Market Price</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="n">
+        <v>108.45</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>LBO Sponsor MOIC</t>
-        </is>
-      </c>
-      <c r="B21" s="26">
-        <f>LBO!B41</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22"/>
+          <t>DCF Implied Price</t>
+        </is>
+      </c>
+      <c r="B21" s="24">
+        <f>DCF!B40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>DCF Upside / (Downside)</t>
+        </is>
+      </c>
+      <c r="B22" s="25">
+        <f>B18/B17-1</f>
+        <v/>
+      </c>
+    </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>LBO Sponsor IRR</t>
+        </is>
+      </c>
+      <c r="B23" s="25">
+        <f>LBO!B40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>LBO Sponsor MOIC</t>
+        </is>
+      </c>
+      <c r="B24" s="26">
+        <f>LBO!B41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Sanity check status</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>0 errors, 2 warnings — see Sanity Checks tab</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>How to use this workbook</t>
         </is>
       </c>
-      <c r="B25" s="22" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="B28" s="22" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>1. Yellow cells (Drivers tab) are the editable inputs — every other tab references them.
 2. Edit any yellow cell to see the model recalculate live.
@@ -1155,25 +1220,183 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30"/>
     <row r="31"/>
     <row r="32"/>
     <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A1:B1"/>
     <mergeCell ref="A26:B33"/>
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36.7109375" customWidth="1" min="1" max="1"/>
+    <col width="18.7109375" customWidth="1" min="2" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>LBO Returns Attribution</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="22" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Decomposition of value created over hold</t>
+        </is>
+      </c>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="22" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>$ Contribution</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>% of Total</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>EBITDA Growth</t>
+        </is>
+      </c>
+      <c r="B5" s="32" t="n">
+        <v>111507462327.3031</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1.335971808635643</v>
+      </c>
+      <c r="D5" s="10">
+        <f> (Exit EBITDA − Entry EBITDA) × Entry Multiple</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Multiple Expansion / (Compression)</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="n">
+        <v>-32408032147.15066</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>-0.388280895451332</v>
+      </c>
+      <c r="D6" s="10">
+        <f> Exit EBITDA × (Exit Mult − Entry Mult)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Debt Paydown + Cash Generation</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="n">
+        <v>4366000457.324661</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.05230908681568902</v>
+      </c>
+      <c r="D7" s="10">
+        <f> ΔDebt + retained cash + recaps</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Total Value Creation</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="n">
+        <v>83465430637.47713</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Sum of above (≈ change in sponsor equity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>How to read this</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="n"/>
+      <c r="C11" s="27" t="n"/>
+      <c r="D11" s="22" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>If EBITDA Growth dominates, the deal works on operational improvement. If Multiple Expansion dominates, the thesis is multiple re-rating — fragile. If Debt Paydown dominates, the deal is a financial-engineering bet — sensitive to interest rate environment and refinancing risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A12:D16"/>
+    <mergeCell ref="A11:D11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1504,7 +1727,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2496,7 +2719,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2995,7 +3218,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3192,7 +3415,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3513,7 +3736,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3687,7 +3910,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3774,7 +3997,7 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>19 fallback / imputation note(s) — see Notes tab.</t>
+          <t>20 fallback / imputation note(s) — see Notes tab.</t>
         </is>
       </c>
     </row>
@@ -3786,13 +4009,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A265"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100.7109375" customWidth="1" min="1" max="1"/>
@@ -3815,1834 +4038,154 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
+          <t>[02:59:25] ⚠ DEMO MODE: data sourced from synthetic test harness, NOT live yfinance.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 87% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 87% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 87% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 88% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 87% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>[16:55:26] ⚠ Terminal value = 87% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 112% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 98% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 94% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 92% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 92% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:26] ⚠ Terminal value = 91% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 130% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 131% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 132% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 134% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 135% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 138% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 105% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 105% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 105% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 105% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 105% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 105% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 94% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 94% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 94% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 94% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 94% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 94% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 88% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 88% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 88% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 88% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 89% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 89% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 85% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] EBITDA margin set via peak_half of trailing 5y (values: [48.7, 44.3, -12.5, 34.6, 46.5]) → 46.5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" s="10" t="inlineStr">
-        <is>
-          <t>[16:55:27] ⚠ Terminal value = 86% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
+          <t>[02:59:26] ⚠ Terminal value = 88% of EV (target &lt;80%). Consider longer explicit forecast or lower terminal growth.</t>
         </is>
       </c>
     </row>
@@ -5674,7 +4217,6 @@
       <c r="B1" s="27" t="n"/>
       <c r="C1" s="22" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -5705,6 +4247,11 @@
       <c r="B5" s="28" t="n">
         <v>1120000000</v>
       </c>
+      <c r="C5" s="54" t="inlineStr">
+        <is>
+          <t>⚠ DEMO  fetched 2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -5713,7 +4260,12 @@
         </is>
       </c>
       <c r="B6" s="29" t="n">
-        <v>668</v>
+        <v>108.45</v>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>⚠ DEMO  fetched 2026-05-08 02:59 UTC</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -5725,6 +4277,11 @@
       <c r="B7" s="30" t="n">
         <v>3850000000</v>
       </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t>⚠ DEMO  fetched 2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -5735,8 +4292,12 @@
       <c r="B8" s="29" t="n">
         <v>1.27</v>
       </c>
-    </row>
-    <row r="9"/>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t>⚠ DEMO  fetched 2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -5753,7 +4314,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="12">
@@ -5851,7 +4412,6 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
@@ -5921,7 +4481,6 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
@@ -5951,7 +4510,6 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
@@ -6030,6 +4588,416 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>DATA SOURCES &amp; FRESHNESS — MU (Micron Technology, Inc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="37" t="inlineStr">
+        <is>
+          <t>Data pulled at</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="37" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>demo/synthetic</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="37" t="inlineStr">
+        <is>
+          <t>Demo / synthetic mode</t>
+        </is>
+      </c>
+      <c r="B5" s="55" t="inlineStr">
+        <is>
+          <t>YES — see warning on Cover</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="inlineStr">
+        <is>
+          <t>Has stale/fallback data?</t>
+        </is>
+      </c>
+      <c r="B6" s="55" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>PER-FIELD PROVENANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="44" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C9" s="44" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>Fetched at</t>
+        </is>
+      </c>
+      <c r="E9" s="44" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>108.4500</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>demo/synthetic</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
+      <c r="E10" s="56" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>shares_out</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1,120,000,000.0000</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>demo/synthetic</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
+      <c r="E11" s="56" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>market_cap</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>121,500,000,000.0000</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>demo/synthetic</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
+      <c r="E12" s="56" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>total_debt</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>13,850,000,000.0000</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>demo/synthetic</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
+      <c r="E13" s="56" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10,000,000,000.0000</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>demo/synthetic</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
+      <c r="E14" s="56" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>enterprise_value</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>125,350,000,000.0000</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>demo/synthetic</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
+      <c r="E15" s="56" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1.2700</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>demo/synthetic</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
+      <c r="E16" s="56" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>dividend_yield</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0.0042</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>demo/synthetic</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-05-08 02:59 UTC</t>
+        </is>
+      </c>
+      <c r="E17" s="56" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="36" t="inlineStr">
+        <is>
+          <t>HOW TO REFRESH AGAINST LIVE DATA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>From the model directory, run:</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   python run_model.py MU</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>yfinance pulls fresh price, shares, debt, beta, and statements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>The freshly-built workbook will replace this one and the banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>above will turn green ('LIVE MARKET DATA — pulled &lt;timestamp&gt;').</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>If yfinance fails or fields are missing, fallbacks are still</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>logged with status='fallback' / 'synthesized' so you can audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>exactly which numbers were inferred vs. reported.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A27:E27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6698,7 +5666,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6866,7 +5834,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7237,7 +6205,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8185,7 +7153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8607,7 +7575,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9269,160 +8237,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="36.7109375" customWidth="1" min="1" max="1"/>
-    <col width="18.7109375" customWidth="1" min="2" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>LBO Returns Attribution</t>
-        </is>
-      </c>
-      <c r="B1" s="27" t="n"/>
-      <c r="C1" s="27" t="n"/>
-      <c r="D1" s="22" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Decomposition of value created over hold</t>
-        </is>
-      </c>
-      <c r="B3" s="27" t="n"/>
-      <c r="C3" s="27" t="n"/>
-      <c r="D3" s="22" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>Driver</t>
-        </is>
-      </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>$ Contribution</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>% of Total</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>EBITDA Growth</t>
-        </is>
-      </c>
-      <c r="B5" s="32" t="n">
-        <v>111507462327.3031</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>1.335971808635643</v>
-      </c>
-      <c r="D5" s="10">
-        <f> (Exit EBITDA − Entry EBITDA) × Entry Multiple</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Multiple Expansion / (Compression)</t>
-        </is>
-      </c>
-      <c r="B6" s="32" t="n">
-        <v>-32408032147.15066</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>-0.388280895451332</v>
-      </c>
-      <c r="D6" s="10">
-        <f> Exit EBITDA × (Exit Mult − Entry Mult)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Debt Paydown + Cash Generation</t>
-        </is>
-      </c>
-      <c r="B7" s="32" t="n">
-        <v>4366000457.324661</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>0.05230908681568902</v>
-      </c>
-      <c r="D7" s="10">
-        <f> ΔDebt + retained cash + recaps</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>Total Value Creation</t>
-        </is>
-      </c>
-      <c r="B8" s="32" t="n">
-        <v>83465430637.47713</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>Sum of above (≈ change in sponsor equity)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>How to read this</t>
-        </is>
-      </c>
-      <c r="B11" s="27" t="n"/>
-      <c r="C11" s="27" t="n"/>
-      <c r="D11" s="22" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>If EBITDA Growth dominates, the deal works on operational improvement. If Multiple Expansion dominates, the thesis is multiple re-rating — fragile. If Debt Paydown dominates, the deal is a financial-engineering bet — sensitive to interest rate environment and refinancing risk.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A12:D16"/>
-    <mergeCell ref="A11:D11"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
MU: live yfinance refresh + 3 SVG charts; v=28
</commit_message>
<xml_diff>
--- a/assets/toolkit/MU_ai_cycle.xlsx
+++ b/assets/toolkit/MU_ai_cycle.xlsx
@@ -913,10 +913,10 @@
     <t>Every fallback or imputation used by the model is logged below.</t>
   </si>
   <si>
-    <t>[20:08:37] EBITDA margin set via peak_half of trailing 5y (values: [54.9, 16.0, 38.2, 49.4]) → 52.2%.</t>
-  </si>
-  <si>
-    <t>[20:08:44] ⚠ EV/EBITDA range 38.0× — peers likely at different cycle positions or business mixes. Median may be misleading; consider tighter peer set.</t>
+    <t>[20:16:04] EBITDA margin set via peak_half of trailing 5y (values: [54.9, 16.0, 38.2, 49.4]) → 52.2%.</t>
+  </si>
+  <si>
+    <t>[20:16:11] ⚠ EV/EBITDA range 38.0× — peers likely at different cycle positions or business mixes. Median may be misleading; consider tighter peer set.</t>
   </si>
 </sst>
 </file>

</xml_diff>